<commit_message>
fix: guard None totalDigits in engine/xsd_model.py's decimal type_display
XSD decimal types that declare fractionDigits but not totalDigits made
_type_display() render the literal string "Decimal (None digits total,
N decimals)" in generated docs. Omit the digits-total clause entirely
when totalDigits is absent instead of interpolating None.

Fixes 18 affected decimal columns in kafe's generated request
data-dictionary (fields.include.bs / TEMPLATE_FIELDS.md /
template_metadata.json / kafe-v4.3.2.xlsx) and 3 fields in
va.include.bs. mikadiv-vib's generated output is unaffected (its
decimal types all declare totalDigits already) - verified by
regenerating and diffing its output.
</commit_message>
<xml_diff>
--- a/kafe/generated/kafe-v4.3.2.xlsx
+++ b/kafe/generated/kafe-v4.3.2.xlsx
@@ -7003,7 +7003,7 @@
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 4 decimals)</t>
+          <t>Decimal (4 decimals)</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
@@ -7013,7 +7013,7 @@
       </c>
       <c r="H3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 4 decimals)</t>
+          <t>Decimal (4 decimals)</t>
         </is>
       </c>
       <c r="I3" s="8" t="inlineStr">
@@ -7043,7 +7043,7 @@
       </c>
       <c r="N3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 4 decimals)</t>
+          <t>Decimal (4 decimals)</t>
         </is>
       </c>
       <c r="O3" s="8" t="inlineStr">
@@ -7068,12 +7068,12 @@
       </c>
       <c r="S3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 2 decimals)</t>
+          <t>Decimal (2 decimals)</t>
         </is>
       </c>
       <c r="T3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 2 decimals)</t>
+          <t>Decimal (2 decimals)</t>
         </is>
       </c>
       <c r="U3" s="8" t="inlineStr">
@@ -7128,7 +7128,7 @@
       </c>
       <c r="AE3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 2 decimals)</t>
+          <t>Decimal (2 decimals)</t>
         </is>
       </c>
       <c r="AF3" s="8" t="inlineStr">
@@ -7143,27 +7143,27 @@
       </c>
       <c r="AH3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 2 decimals)</t>
+          <t>Decimal (2 decimals)</t>
         </is>
       </c>
       <c r="AI3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 4 decimals)</t>
+          <t>Decimal (4 decimals)</t>
         </is>
       </c>
       <c r="AJ3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 4 decimals)</t>
+          <t>Decimal (4 decimals)</t>
         </is>
       </c>
       <c r="AK3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 4 decimals)</t>
+          <t>Decimal (4 decimals)</t>
         </is>
       </c>
       <c r="AL3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 4 decimals)</t>
+          <t>Decimal (4 decimals)</t>
         </is>
       </c>
       <c r="AM3" s="8" t="inlineStr">
@@ -7173,7 +7173,7 @@
       </c>
       <c r="AN3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 4 decimals)</t>
+          <t>Decimal (4 decimals)</t>
         </is>
       </c>
       <c r="AO3" s="8" t="inlineStr">
@@ -7188,7 +7188,7 @@
       </c>
       <c r="AQ3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 4 decimals)</t>
+          <t>Decimal (4 decimals)</t>
         </is>
       </c>
       <c r="AR3" s="8" t="inlineStr">
@@ -7203,7 +7203,7 @@
       </c>
       <c r="AT3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 4 decimals)</t>
+          <t>Decimal (4 decimals)</t>
         </is>
       </c>
     </row>
@@ -7660,7 +7660,7 @@
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 4 decimals)</t>
+          <t>Decimal (4 decimals)</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
@@ -7941,7 +7941,7 @@
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 4 decimals)</t>
+          <t>Decimal (4 decimals)</t>
         </is>
       </c>
       <c r="F3" s="8" t="inlineStr">
@@ -7951,7 +7951,7 @@
       </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 4 decimals)</t>
+          <t>Decimal (4 decimals)</t>
         </is>
       </c>
       <c r="H3" s="8" t="inlineStr">
@@ -7976,7 +7976,7 @@
       </c>
       <c r="L3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 4 decimals)</t>
+          <t>Decimal (4 decimals)</t>
         </is>
       </c>
       <c r="M3" s="8" t="inlineStr">

</xml_diff>

<commit_message>
fix: guard None totalDigits in engine/xsd_model.py's decimal type_display (#13)
XSD decimal types that declare fractionDigits but not totalDigits made
_type_display() render the literal string "Decimal (None digits total,
N decimals)" in generated docs. Omit the digits-total clause entirely
when totalDigits is absent instead of interpolating None.

Fixes 18 affected decimal columns in kafe's generated request
data-dictionary (fields.include.bs / TEMPLATE_FIELDS.md /
template_metadata.json / kafe-v4.3.2.xlsx) and 3 fields in
va.include.bs. mikadiv-vib's generated output is unaffected (its
decimal types all declare totalDigits already) - verified by
regenerating and diffing its output.
</commit_message>
<xml_diff>
--- a/kafe/generated/kafe-v4.3.2.xlsx
+++ b/kafe/generated/kafe-v4.3.2.xlsx
@@ -7003,7 +7003,7 @@
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 4 decimals)</t>
+          <t>Decimal (4 decimals)</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
@@ -7013,7 +7013,7 @@
       </c>
       <c r="H3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 4 decimals)</t>
+          <t>Decimal (4 decimals)</t>
         </is>
       </c>
       <c r="I3" s="8" t="inlineStr">
@@ -7043,7 +7043,7 @@
       </c>
       <c r="N3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 4 decimals)</t>
+          <t>Decimal (4 decimals)</t>
         </is>
       </c>
       <c r="O3" s="8" t="inlineStr">
@@ -7068,12 +7068,12 @@
       </c>
       <c r="S3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 2 decimals)</t>
+          <t>Decimal (2 decimals)</t>
         </is>
       </c>
       <c r="T3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 2 decimals)</t>
+          <t>Decimal (2 decimals)</t>
         </is>
       </c>
       <c r="U3" s="8" t="inlineStr">
@@ -7128,7 +7128,7 @@
       </c>
       <c r="AE3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 2 decimals)</t>
+          <t>Decimal (2 decimals)</t>
         </is>
       </c>
       <c r="AF3" s="8" t="inlineStr">
@@ -7143,27 +7143,27 @@
       </c>
       <c r="AH3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 2 decimals)</t>
+          <t>Decimal (2 decimals)</t>
         </is>
       </c>
       <c r="AI3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 4 decimals)</t>
+          <t>Decimal (4 decimals)</t>
         </is>
       </c>
       <c r="AJ3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 4 decimals)</t>
+          <t>Decimal (4 decimals)</t>
         </is>
       </c>
       <c r="AK3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 4 decimals)</t>
+          <t>Decimal (4 decimals)</t>
         </is>
       </c>
       <c r="AL3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 4 decimals)</t>
+          <t>Decimal (4 decimals)</t>
         </is>
       </c>
       <c r="AM3" s="8" t="inlineStr">
@@ -7173,7 +7173,7 @@
       </c>
       <c r="AN3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 4 decimals)</t>
+          <t>Decimal (4 decimals)</t>
         </is>
       </c>
       <c r="AO3" s="8" t="inlineStr">
@@ -7188,7 +7188,7 @@
       </c>
       <c r="AQ3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 4 decimals)</t>
+          <t>Decimal (4 decimals)</t>
         </is>
       </c>
       <c r="AR3" s="8" t="inlineStr">
@@ -7203,7 +7203,7 @@
       </c>
       <c r="AT3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 4 decimals)</t>
+          <t>Decimal (4 decimals)</t>
         </is>
       </c>
     </row>
@@ -7660,7 +7660,7 @@
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 4 decimals)</t>
+          <t>Decimal (4 decimals)</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
@@ -7941,7 +7941,7 @@
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 4 decimals)</t>
+          <t>Decimal (4 decimals)</t>
         </is>
       </c>
       <c r="F3" s="8" t="inlineStr">
@@ -7951,7 +7951,7 @@
       </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 4 decimals)</t>
+          <t>Decimal (4 decimals)</t>
         </is>
       </c>
       <c r="H3" s="8" t="inlineStr">
@@ -7976,7 +7976,7 @@
       </c>
       <c r="L3" s="8" t="inlineStr">
         <is>
-          <t>Decimal (None digits total, 4 decimals)</t>
+          <t>Decimal (4 decimals)</t>
         </is>
       </c>
       <c r="M3" s="8" t="inlineStr">

</xml_diff>